<commit_message>
Updated Project for stability
</commit_message>
<xml_diff>
--- a/COST.xlsx
+++ b/COST.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{128C6530-8463-4D0F-83BE-57B4B8047B1A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{38C798D6-8780-4836-BB4A-1EF7E31E707D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="21840" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="COST" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1060" uniqueCount="440">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1284" uniqueCount="522">
   <si>
     <t>S.No</t>
   </si>
@@ -982,9 +982,6 @@
     <t>SHROUD STRG/COL LWR + KEY</t>
   </si>
   <si>
-    <t>51</t>
-  </si>
-  <si>
     <t>HOUSING S A STD SU2i R C LH HOUSING S A STD SU2I R C RH</t>
   </si>
   <si>
@@ -1340,13 +1337,262 @@
   </si>
   <si>
     <t>415</t>
+  </si>
+  <si>
+    <t>SHIELD  COVER  FRT  SEAT  INR  RH  PWR NNB</t>
+  </si>
+  <si>
+    <t>S/COVER FRT SEAT OTR LH MNL H/ADJ LHD; S/COVER FRT CUSH OTR RH MNL  YGN</t>
+  </si>
+  <si>
+    <t>PS7IRDE</t>
+  </si>
+  <si>
+    <t>PNL ASSY-CRASH PAD LWR D/SIDE TTX RHD LHTX</t>
+  </si>
+  <si>
+    <t>COVER-GLOVE BOX LHD TTX</t>
+  </si>
+  <si>
+    <t>SHIELD COVER FRT SEAT OTR LH H/ADJ TTX</t>
+  </si>
+  <si>
+    <t>TRIM LUGG TRAY COVERLH/RH NNB</t>
+  </si>
+  <si>
+    <t>SHIELD COVER FR SEAT INR LH PWR NNB</t>
+  </si>
+  <si>
+    <t>SHIELD COVER FR SEAT INR LH PWR YGN</t>
+  </si>
+  <si>
+    <t>SHIELD COVER FRT SEAT OTR RH STD TTX</t>
+  </si>
+  <si>
+    <t>PNL ASSY-CRASH PAD LWR D/SIDE LHD UMG</t>
+  </si>
+  <si>
+    <t>368</t>
+  </si>
+  <si>
+    <t>KNOB FR SEAT RECL RH NNB</t>
+  </si>
+  <si>
+    <t>PNL ASSY-CRASH PAD LWR D SIDE YPK RHD LHYP</t>
+  </si>
+  <si>
+    <t>S/COVER FRT CUSH OTR RH MNL UMG</t>
+  </si>
+  <si>
+    <t>KNOB FR SEAT RECL LH NNB</t>
+  </si>
+  <si>
+    <t>LQ2I HOUSING124W</t>
+  </si>
+  <si>
+    <t>KNOB ASSY FRT SEAT H /ADJ RH NNB</t>
+  </si>
+  <si>
+    <t>COVER COOL BOX LHD</t>
+  </si>
+  <si>
+    <t>AI3/SUVE</t>
+  </si>
+  <si>
+    <t>61</t>
+  </si>
+  <si>
+    <t>SHIELD COVER FRT SEAT OTR STD LH/H.RH NNB</t>
+  </si>
+  <si>
+    <t>SHIELD COVER FRT SEAT OTR STD LH/H.RH NBY</t>
+  </si>
+  <si>
+    <t>SHIELD COVER FRT SEAT OTR HEIGHT LH NNB</t>
+  </si>
+  <si>
+    <t>SHIELD COVER FRT SEAT OTR HEIGHT LH T9Y</t>
+  </si>
+  <si>
+    <t>SHIELD COVER FRT SEAT OTR STD LH T9Y</t>
+  </si>
+  <si>
+    <t>SU2I/BI3</t>
+  </si>
+  <si>
+    <t>S/COVER FRT SEAT OTR LH H.ADJ/RH MNL NNB</t>
+  </si>
+  <si>
+    <t>75</t>
+  </si>
+  <si>
+    <t>S/COVER FRT SEAT OTR LH MNL/RH H.ADJ YGN</t>
+  </si>
+  <si>
+    <t>78</t>
+  </si>
+  <si>
+    <t>HOUSING-GLOVE BOX LHD MMH</t>
+  </si>
+  <si>
+    <t>DUCT DEFROSTER REAR LHD</t>
+  </si>
+  <si>
+    <t>121</t>
+  </si>
+  <si>
+    <t>HOUSING-GLOVE BOX RHD #3 MMH</t>
+  </si>
+  <si>
+    <t>HOUSING-GLOVE BOX RHD #3 TTX</t>
+  </si>
+  <si>
+    <t>HOUSING-GLOVE BOX RHD #3 YPK</t>
+  </si>
+  <si>
+    <t>TRIM-LUGG SIDE  SPEAKER RH YGN</t>
+  </si>
+  <si>
+    <t>365</t>
+  </si>
+  <si>
+    <t>TRIM-LUGG SIDE W/O SPKR RH YGN</t>
+  </si>
+  <si>
+    <t>TRIM LUGGAGE SIDE LH NNB</t>
+  </si>
+  <si>
+    <t>385</t>
+  </si>
+  <si>
+    <t>TRIM LUGGAGE SIDE LH YGN</t>
+  </si>
+  <si>
+    <t>S/COVER FRT CUSH OTR RH MNL H/ADJ RHD YGN</t>
+  </si>
+  <si>
+    <t>SHIELD  COVER  FRT  SEAT  INR  RH  PWR WDN</t>
+  </si>
+  <si>
+    <t>Santhosh</t>
+  </si>
+  <si>
+    <t>994654354654</t>
+  </si>
+  <si>
+    <t>LEVER ASSY FRT SEAT H/ADJ RH NBY</t>
+  </si>
+  <si>
+    <t>Ai3SUV</t>
+  </si>
+  <si>
+    <t>PNL-ASSY C/PAD LWR DRIVER SIDE RHD TTX</t>
+  </si>
+  <si>
+    <t>PNL-ASSY C/PAD LWR DRIVER SIDE RHD YPK</t>
+  </si>
+  <si>
+    <t>66</t>
+  </si>
+  <si>
+    <t>S/COVER FRT SEAT OTR LH MNL/RH H.ADJ WDN</t>
+  </si>
+  <si>
+    <t>86</t>
+  </si>
+  <si>
+    <t>SHIELD COVER -FR SEAT OTR PWR RH YGN</t>
+  </si>
+  <si>
+    <t>HOUSING REAR COMBI OPT LH/RH</t>
+  </si>
+  <si>
+    <t>SIDE SILL LH/RH</t>
+  </si>
+  <si>
+    <t>TRIM-LUGG SIDE LH SUB WOOFER RDE WDN</t>
+  </si>
+  <si>
+    <t>382</t>
+  </si>
+  <si>
+    <t>PNL C/PAD LWR RHD NO HOLE T9Y</t>
+  </si>
+  <si>
+    <t>18</t>
+  </si>
+  <si>
+    <t>DR ASSY-PASSENGER AIRBAG RHD #1</t>
+  </si>
+  <si>
+    <t>PNL ASSY-CRASH PAD LWR D/SIDE YPK RHD      LLYP</t>
+  </si>
+  <si>
+    <t>Ai3/SUVPE</t>
+  </si>
+  <si>
+    <t>PNL ASSY-CRASH PAD LWR D/SIDE MMH RHD LHTX</t>
+  </si>
+  <si>
+    <t>83</t>
+  </si>
+  <si>
+    <t>SHIELD COVER FRT SEAT OTR LH STD/ RH       H/ADJ T9Y</t>
+  </si>
+  <si>
+    <t>S/COVER FRT SEAT OTR LH H.ADJ/RH MNL        NNB</t>
+  </si>
+  <si>
+    <t>S/COVER OTR FRT SEAT OTR LH MNL/RH.H ADJ  NNB</t>
+  </si>
+  <si>
+    <t>LEVER ASSY-FR SEAT HGT_ADJM, RH</t>
+  </si>
+  <si>
+    <t>SHIELD COVER FRT SEAT OTR LH STD QXI</t>
+  </si>
+  <si>
+    <t>SU2i/BN7i/Bi3</t>
+  </si>
+  <si>
+    <t>PNL ASSY-CRASH PAD LWR D/SIDE +SSB NNB LHD NNB</t>
+  </si>
+  <si>
+    <t>S/COVER FRT SEAT OTR LH MNL; S/COVER FRT SEAT OTR LH MNL H/ADJ LHD YGN</t>
+  </si>
+  <si>
+    <t>HOUSING BN7I DRL PSTN RH</t>
+  </si>
+  <si>
+    <t>SHIELD COVER-2ND CUSH OTR LH; SHIELD COVER 2ND CUSH OTR RH WDN</t>
+  </si>
+  <si>
+    <t>HOUSING BN7I DRL PSTN LH</t>
+  </si>
+  <si>
+    <t>KNOB ASSY FRT SEAT H /ADJ LH YGN</t>
+  </si>
+  <si>
+    <t>PNL FR DR MAIN TRIM LH NNB</t>
+  </si>
+  <si>
+    <t>PS7IFL</t>
+  </si>
+  <si>
+    <t>HOUSING 72W</t>
+  </si>
+  <si>
+    <t>SHILD CVR INR LH HT ADJ; SHILD CVR INR  RH NNB</t>
+  </si>
+  <si>
+    <t>GSPE MOULDING ASSY-SIDE SILL,LH</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="20" x14ac:knownFonts="1">
+  <fonts count="28" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1471,6 +1717,62 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="8"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -1520,7 +1822,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1586,6 +1888,30 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="19" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="21" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="24" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="27" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1744,8 +2070,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table1" displayName="Table1" ref="A1:D437" totalsRowShown="0" headerRowDxfId="5" dataDxfId="4">
-  <autoFilter ref="A1:D437" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table1" displayName="Table1" ref="A1:D528" totalsRowShown="0" headerRowDxfId="5" dataDxfId="4">
+  <autoFilter ref="A1:D528" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:D56">
     <sortCondition ref="C1:C56"/>
   </sortState>
@@ -2022,7 +2348,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D437"/>
+  <dimension ref="A1:D528"/>
   <sheetFormatPr defaultColWidth="52.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="7.42578125" style="1" bestFit="1" customWidth="1"/>
@@ -2084,8 +2410,8 @@
       <c r="C4" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="D4" s="3" t="s">
-        <v>9</v>
+      <c r="D4" s="3">
+        <v>76</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
@@ -2224,8 +2550,8 @@
       <c r="C14" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="D14" s="3" t="s">
-        <v>25</v>
+      <c r="D14" s="3">
+        <v>48</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
@@ -2644,8 +2970,8 @@
       <c r="C44" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="D44" s="3" t="s">
-        <v>67</v>
+      <c r="D44" s="3">
+        <v>233</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.25">
@@ -2855,7 +3181,7 @@
         <v>87</v>
       </c>
       <c r="D59" s="5">
-        <v>201</v>
+        <v>202</v>
       </c>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.25">
@@ -2981,7 +3307,7 @@
         <v>101</v>
       </c>
       <c r="D68" s="5">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.25">
@@ -3092,8 +3418,8 @@
       <c r="C76" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="D76" s="5">
-        <v>82</v>
+      <c r="D76" s="5" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.25">
@@ -3120,8 +3446,8 @@
       <c r="C78" s="4" t="s">
         <v>115</v>
       </c>
-      <c r="D78" s="5" t="s">
-        <v>45</v>
+      <c r="D78" s="5">
+        <v>82</v>
       </c>
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.25">
@@ -5011,7 +5337,7 @@
         <v>250</v>
       </c>
       <c r="D213" s="5">
-        <v>20</v>
+        <v>17</v>
       </c>
     </row>
     <row r="214" spans="1:4" x14ac:dyDescent="0.25">
@@ -5248,8 +5574,8 @@
       <c r="C230" s="4" t="s">
         <v>266</v>
       </c>
-      <c r="D230" s="5" t="s">
-        <v>267</v>
+      <c r="D230" s="5">
+        <v>59</v>
       </c>
     </row>
     <row r="231" spans="1:4" x14ac:dyDescent="0.25">
@@ -5668,8 +5994,8 @@
       <c r="C260" s="4" t="s">
         <v>291</v>
       </c>
-      <c r="D260" s="5" t="s">
-        <v>163</v>
+      <c r="D260" s="5">
+        <v>81</v>
       </c>
     </row>
     <row r="261" spans="1:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -5780,8 +6106,8 @@
       <c r="C268" s="4" t="s">
         <v>295</v>
       </c>
-      <c r="D268" s="5" t="s">
-        <v>296</v>
+      <c r="D268" s="5">
+        <v>130</v>
       </c>
     </row>
     <row r="269" spans="1:4" x14ac:dyDescent="0.25">
@@ -5808,8 +6134,8 @@
       <c r="C270" s="4" t="s">
         <v>298</v>
       </c>
-      <c r="D270" s="5">
-        <v>207</v>
+      <c r="D270" s="5" t="s">
+        <v>283</v>
       </c>
     </row>
     <row r="271" spans="1:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -5990,8 +6316,8 @@
       <c r="C283" s="9" t="s">
         <v>310</v>
       </c>
-      <c r="D283" s="10" t="s">
-        <v>67</v>
+      <c r="D283" s="10">
+        <v>233</v>
       </c>
     </row>
     <row r="284" spans="1:4" x14ac:dyDescent="0.25">
@@ -6200,8 +6526,8 @@
       <c r="C298" s="4" t="s">
         <v>319</v>
       </c>
-      <c r="D298" s="5" t="s">
-        <v>320</v>
+      <c r="D298" s="5">
+        <v>51</v>
       </c>
     </row>
     <row r="299" spans="1:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -6212,7 +6538,7 @@
         <v>93</v>
       </c>
       <c r="C299" s="4" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="D299" s="5" t="s">
         <v>61</v>
@@ -6226,7 +6552,7 @@
         <v>93</v>
       </c>
       <c r="C300" s="4" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="D300" s="5" t="s">
         <v>61</v>
@@ -6240,7 +6566,7 @@
         <v>83</v>
       </c>
       <c r="C301" s="4" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="D301" s="5">
         <v>123</v>
@@ -6251,7 +6577,7 @@
         <v>301</v>
       </c>
       <c r="B302" s="4" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="C302" s="4" t="s">
         <v>47</v>
@@ -6265,7 +6591,7 @@
         <v>302</v>
       </c>
       <c r="B303" s="4" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="C303" s="4" t="s">
         <v>317</v>
@@ -6282,7 +6608,7 @@
         <v>240</v>
       </c>
       <c r="C304" s="4" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="D304" s="5">
         <v>67</v>
@@ -6296,7 +6622,7 @@
         <v>50</v>
       </c>
       <c r="C305" s="4" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="D305" s="5">
         <v>84</v>
@@ -6310,7 +6636,7 @@
         <v>240</v>
       </c>
       <c r="C306" s="4" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="D306" s="5">
         <v>67</v>
@@ -6324,7 +6650,7 @@
         <v>240</v>
       </c>
       <c r="C307" s="4" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="D307" s="5">
         <v>67</v>
@@ -6338,7 +6664,7 @@
         <v>240</v>
       </c>
       <c r="C308" s="4" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="D308" s="5">
         <v>67</v>
@@ -6349,10 +6675,10 @@
         <v>308</v>
       </c>
       <c r="B309" s="4" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="C309" s="4" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="D309" s="5">
         <v>82</v>
@@ -6366,7 +6692,7 @@
         <v>50</v>
       </c>
       <c r="C310" s="4" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="D310" s="5">
         <v>13</v>
@@ -6380,7 +6706,7 @@
         <v>240</v>
       </c>
       <c r="C311" s="4" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="D311" s="5">
         <v>67</v>
@@ -6394,7 +6720,7 @@
         <v>50</v>
       </c>
       <c r="C312" s="4" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="D312" s="5">
         <v>323</v>
@@ -6408,7 +6734,7 @@
         <v>240</v>
       </c>
       <c r="C313" s="4" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="D313" s="5">
         <v>19</v>
@@ -6422,7 +6748,7 @@
         <v>240</v>
       </c>
       <c r="C314" s="4" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="D314" s="5">
         <v>19</v>
@@ -6436,7 +6762,7 @@
         <v>13</v>
       </c>
       <c r="C315" s="4" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="D315" s="5">
         <v>70</v>
@@ -6450,7 +6776,7 @@
         <v>4</v>
       </c>
       <c r="C316" s="4" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="D316" s="5">
         <v>211</v>
@@ -6461,10 +6787,10 @@
         <v>316</v>
       </c>
       <c r="B317" s="4" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="C317" s="4" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="D317" s="5">
         <v>67</v>
@@ -6475,7 +6801,7 @@
         <v>317</v>
       </c>
       <c r="B318" s="4" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="C318" s="4" t="s">
         <v>24</v>
@@ -6492,10 +6818,10 @@
         <v>4</v>
       </c>
       <c r="C319" s="12" t="s">
+        <v>339</v>
+      </c>
+      <c r="D319" s="13" t="s">
         <v>340</v>
-      </c>
-      <c r="D319" s="13" t="s">
-        <v>341</v>
       </c>
     </row>
     <row r="320" spans="1:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -6506,7 +6832,7 @@
         <v>83</v>
       </c>
       <c r="C320" s="4" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="D320" s="5" t="s">
         <v>56</v>
@@ -6520,7 +6846,7 @@
         <v>83</v>
       </c>
       <c r="C321" s="4" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="D321" s="5" t="s">
         <v>56</v>
@@ -6531,7 +6857,7 @@
         <v>321</v>
       </c>
       <c r="B322" s="4" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="C322" s="4" t="s">
         <v>188</v>
@@ -6548,7 +6874,7 @@
         <v>62</v>
       </c>
       <c r="C323" s="4" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="D323" s="5" t="s">
         <v>56</v>
@@ -6576,7 +6902,7 @@
         <v>93</v>
       </c>
       <c r="C325" s="4" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="D325" s="5" t="s">
         <v>61</v>
@@ -6590,7 +6916,7 @@
         <v>121</v>
       </c>
       <c r="C326" s="4" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="D326" s="5">
         <v>67</v>
@@ -6604,7 +6930,7 @@
         <v>113</v>
       </c>
       <c r="C327" s="4" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="D327" s="5">
         <v>14</v>
@@ -6615,10 +6941,10 @@
         <v>327</v>
       </c>
       <c r="B328" s="4" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="C328" s="4" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="D328" s="5">
         <v>82</v>
@@ -6646,7 +6972,7 @@
         <v>4</v>
       </c>
       <c r="C330" s="4" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="D330" s="5" t="s">
         <v>119</v>
@@ -6674,7 +7000,7 @@
         <v>83</v>
       </c>
       <c r="C332" s="4" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="D332" s="5" t="s">
         <v>36</v>
@@ -6730,7 +7056,7 @@
         <v>281</v>
       </c>
       <c r="C336" s="4" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="D336" s="5" t="s">
         <v>61</v>
@@ -6744,7 +7070,7 @@
         <v>93</v>
       </c>
       <c r="C337" s="4" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="D337" s="5" t="s">
         <v>61</v>
@@ -6758,10 +7084,10 @@
         <v>91</v>
       </c>
       <c r="C338" s="4" t="s">
-        <v>354</v>
-      </c>
-      <c r="D338" s="5" t="s">
-        <v>260</v>
+        <v>353</v>
+      </c>
+      <c r="D338" s="5">
+        <v>124</v>
       </c>
     </row>
     <row r="339" spans="1:4" x14ac:dyDescent="0.25">
@@ -6772,7 +7098,7 @@
         <v>103</v>
       </c>
       <c r="C339" s="4" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="D339" s="5">
         <v>340</v>
@@ -6783,7 +7109,7 @@
         <v>339</v>
       </c>
       <c r="B340" s="4" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="C340" s="4" t="s">
         <v>82</v>
@@ -6800,7 +7126,7 @@
         <v>113</v>
       </c>
       <c r="C341" s="4" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="D341" s="5" t="s">
         <v>161</v>
@@ -6814,7 +7140,7 @@
         <v>307</v>
       </c>
       <c r="C342" s="4" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="D342" s="5" t="s">
         <v>119</v>
@@ -6828,7 +7154,7 @@
         <v>307</v>
       </c>
       <c r="C343" s="4" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="D343" s="5" t="s">
         <v>119</v>
@@ -6839,10 +7165,10 @@
         <v>343</v>
       </c>
       <c r="B344" s="4" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="C344" s="4" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="D344" s="5">
         <v>67</v>
@@ -6884,7 +7210,7 @@
         <v>221</v>
       </c>
       <c r="C347" s="4" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="D347" s="5">
         <v>13</v>
@@ -6895,10 +7221,10 @@
         <v>347</v>
       </c>
       <c r="B348" s="4" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="C348" s="4" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="D348" s="5">
         <v>123</v>
@@ -6926,7 +7252,7 @@
         <v>83</v>
       </c>
       <c r="C350" s="4" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="D350" s="5">
         <v>45</v>
@@ -6951,7 +7277,7 @@
         <v>351</v>
       </c>
       <c r="B352" s="15" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="C352" s="15" t="s">
         <v>315</v>
@@ -6968,7 +7294,7 @@
         <v>113</v>
       </c>
       <c r="C353" s="15" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="D353" s="16" t="s">
         <v>163</v>
@@ -6982,7 +7308,7 @@
         <v>248</v>
       </c>
       <c r="C354" s="15" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="D354" s="16">
         <v>67</v>
@@ -6996,10 +7322,10 @@
         <v>135</v>
       </c>
       <c r="C355" s="15" t="s">
+        <v>364</v>
+      </c>
+      <c r="D355" s="16" t="s">
         <v>365</v>
-      </c>
-      <c r="D355" s="16" t="s">
-        <v>366</v>
       </c>
     </row>
     <row r="356" spans="1:4" x14ac:dyDescent="0.25">
@@ -7010,7 +7336,7 @@
         <v>4</v>
       </c>
       <c r="C356" s="15" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="D356" s="16" t="s">
         <v>195</v>
@@ -7021,10 +7347,10 @@
         <v>356</v>
       </c>
       <c r="B357" s="15" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="C357" s="15" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="D357" s="16" t="s">
         <v>163</v>
@@ -7052,7 +7378,7 @@
         <v>7</v>
       </c>
       <c r="C359" s="4" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="D359" s="5">
         <v>81</v>
@@ -7066,7 +7392,7 @@
         <v>141</v>
       </c>
       <c r="C360" s="4" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="D360" s="5">
         <v>81</v>
@@ -7080,7 +7406,7 @@
         <v>240</v>
       </c>
       <c r="C361" s="4" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="D361" s="5">
         <v>67</v>
@@ -7094,7 +7420,7 @@
         <v>7</v>
       </c>
       <c r="C362" s="4" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="D362" s="5" t="s">
         <v>163</v>
@@ -7108,7 +7434,7 @@
         <v>4</v>
       </c>
       <c r="C363" s="4" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="D363" s="5">
         <v>313</v>
@@ -7119,10 +7445,10 @@
         <v>363</v>
       </c>
       <c r="B364" s="4" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="C364" s="4" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="D364" s="5">
         <v>22</v>
@@ -7150,7 +7476,7 @@
         <v>113</v>
       </c>
       <c r="C366" s="4" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="D366" s="5">
         <v>81</v>
@@ -7161,10 +7487,10 @@
         <v>366</v>
       </c>
       <c r="B367" s="4" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="C367" s="4" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="D367" s="5">
         <v>81</v>
@@ -7178,7 +7504,7 @@
         <v>4</v>
       </c>
       <c r="C368" s="4" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="D368" s="5">
         <v>302</v>
@@ -7192,7 +7518,7 @@
         <v>4</v>
       </c>
       <c r="C369" s="4" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="D369" s="5">
         <v>128</v>
@@ -7220,7 +7546,7 @@
         <v>246</v>
       </c>
       <c r="C371" s="18" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="D371" s="19">
         <v>67</v>
@@ -7231,7 +7557,7 @@
         <v>371</v>
       </c>
       <c r="B372" s="4" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="C372" s="4" t="s">
         <v>316</v>
@@ -7248,7 +7574,7 @@
         <v>240</v>
       </c>
       <c r="C373" s="4" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="D373" s="5">
         <v>67</v>
@@ -7259,10 +7585,10 @@
         <v>373</v>
       </c>
       <c r="B374" s="4" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="C374" s="4" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="D374" s="5">
         <v>67</v>
@@ -7290,10 +7616,10 @@
         <v>240</v>
       </c>
       <c r="C376" s="4" t="s">
-        <v>379</v>
-      </c>
-      <c r="D376" s="5" t="s">
-        <v>56</v>
+        <v>378</v>
+      </c>
+      <c r="D376" s="5">
+        <v>67</v>
       </c>
     </row>
     <row r="377" spans="1:4" x14ac:dyDescent="0.25">
@@ -7304,7 +7630,7 @@
         <v>13</v>
       </c>
       <c r="C377" s="4" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="D377" s="5">
         <v>121</v>
@@ -7318,7 +7644,7 @@
         <v>113</v>
       </c>
       <c r="C378" s="4" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="D378" s="5">
         <v>22</v>
@@ -7346,7 +7672,7 @@
         <v>13</v>
       </c>
       <c r="C380" s="4" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="D380" s="5">
         <v>124</v>
@@ -7360,7 +7686,7 @@
         <v>37</v>
       </c>
       <c r="C381" s="4" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="D381" s="5">
         <v>382</v>
@@ -7402,7 +7728,7 @@
         <v>227</v>
       </c>
       <c r="C384" s="4" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="D384" s="5">
         <v>369</v>
@@ -7430,7 +7756,7 @@
         <v>240</v>
       </c>
       <c r="C386" s="4" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="D386" s="5">
         <v>67</v>
@@ -7444,7 +7770,7 @@
         <v>83</v>
       </c>
       <c r="C387" s="4" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="D387" s="5">
         <v>45</v>
@@ -7483,13 +7809,13 @@
         <v>389</v>
       </c>
       <c r="B390" s="4" t="s">
+        <v>385</v>
+      </c>
+      <c r="C390" s="4" t="s">
         <v>386</v>
       </c>
-      <c r="C390" s="4" t="s">
+      <c r="D390" s="5" t="s">
         <v>387</v>
-      </c>
-      <c r="D390" s="5" t="s">
-        <v>388</v>
       </c>
     </row>
     <row r="391" spans="1:4" x14ac:dyDescent="0.25">
@@ -7497,13 +7823,13 @@
         <v>390</v>
       </c>
       <c r="B391" s="4" t="s">
+        <v>388</v>
+      </c>
+      <c r="C391" s="4" t="s">
         <v>389</v>
       </c>
-      <c r="C391" s="4" t="s">
+      <c r="D391" s="5" t="s">
         <v>390</v>
-      </c>
-      <c r="D391" s="5" t="s">
-        <v>391</v>
       </c>
     </row>
     <row r="392" spans="1:4" x14ac:dyDescent="0.25">
@@ -7514,10 +7840,10 @@
         <v>111</v>
       </c>
       <c r="C392" s="4" t="s">
+        <v>391</v>
+      </c>
+      <c r="D392" s="5" t="s">
         <v>392</v>
-      </c>
-      <c r="D392" s="5" t="s">
-        <v>393</v>
       </c>
     </row>
     <row r="393" spans="1:4" x14ac:dyDescent="0.25">
@@ -7528,10 +7854,10 @@
         <v>83</v>
       </c>
       <c r="C393" s="4" t="s">
+        <v>393</v>
+      </c>
+      <c r="D393" s="5" t="s">
         <v>394</v>
-      </c>
-      <c r="D393" s="5" t="s">
-        <v>395</v>
       </c>
     </row>
     <row r="394" spans="1:4" x14ac:dyDescent="0.25">
@@ -7542,10 +7868,10 @@
         <v>83</v>
       </c>
       <c r="C394" s="4" t="s">
+        <v>395</v>
+      </c>
+      <c r="D394" s="5" t="s">
         <v>396</v>
-      </c>
-      <c r="D394" s="5" t="s">
-        <v>397</v>
       </c>
     </row>
     <row r="395" spans="1:4" x14ac:dyDescent="0.25">
@@ -7553,10 +7879,10 @@
         <v>394</v>
       </c>
       <c r="B395" s="4" t="s">
+        <v>397</v>
+      </c>
+      <c r="C395" s="4" t="s">
         <v>398</v>
-      </c>
-      <c r="C395" s="4" t="s">
-        <v>399</v>
       </c>
       <c r="D395" s="5" t="s">
         <v>45</v>
@@ -7570,7 +7896,7 @@
         <v>83</v>
       </c>
       <c r="C396" s="4" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="D396" s="5" t="s">
         <v>9</v>
@@ -7584,10 +7910,10 @@
         <v>93</v>
       </c>
       <c r="C397" s="4" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="D397" s="5" t="s">
-        <v>280</v>
+        <v>459</v>
       </c>
     </row>
     <row r="398" spans="1:4" x14ac:dyDescent="0.25">
@@ -7598,10 +7924,10 @@
         <v>116</v>
       </c>
       <c r="C398" s="4" t="s">
+        <v>401</v>
+      </c>
+      <c r="D398" s="5" t="s">
         <v>402</v>
-      </c>
-      <c r="D398" s="5" t="s">
-        <v>403</v>
       </c>
     </row>
     <row r="399" spans="1:4" x14ac:dyDescent="0.25">
@@ -7609,10 +7935,10 @@
         <v>398</v>
       </c>
       <c r="B399" s="4" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="C399" s="4" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="D399" s="5" t="s">
         <v>118</v>
@@ -7626,7 +7952,7 @@
         <v>91</v>
       </c>
       <c r="C400" s="4" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="D400" s="5" t="s">
         <v>56</v>
@@ -7640,10 +7966,10 @@
         <v>93</v>
       </c>
       <c r="C401" s="4" t="s">
+        <v>405</v>
+      </c>
+      <c r="D401" s="5" t="s">
         <v>406</v>
-      </c>
-      <c r="D401" s="5" t="s">
-        <v>407</v>
       </c>
     </row>
     <row r="402" spans="1:4" x14ac:dyDescent="0.25">
@@ -7654,10 +7980,10 @@
         <v>93</v>
       </c>
       <c r="C402" s="4" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="D402" s="5" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
     </row>
     <row r="403" spans="1:4" x14ac:dyDescent="0.25">
@@ -7668,10 +7994,10 @@
         <v>91</v>
       </c>
       <c r="C403" s="4" t="s">
-        <v>409</v>
-      </c>
-      <c r="D403" s="5" t="s">
-        <v>260</v>
+        <v>408</v>
+      </c>
+      <c r="D403" s="5">
+        <v>124</v>
       </c>
     </row>
     <row r="404" spans="1:4" x14ac:dyDescent="0.25">
@@ -7682,7 +8008,7 @@
         <v>83</v>
       </c>
       <c r="C404" s="4" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="D404" s="5" t="s">
         <v>218</v>
@@ -7696,7 +8022,7 @@
         <v>83</v>
       </c>
       <c r="C405" s="4" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="D405" s="5" t="s">
         <v>218</v>
@@ -7710,10 +8036,10 @@
         <v>116</v>
       </c>
       <c r="C406" s="4" t="s">
+        <v>411</v>
+      </c>
+      <c r="D406" s="5" t="s">
         <v>412</v>
-      </c>
-      <c r="D406" s="5" t="s">
-        <v>413</v>
       </c>
     </row>
     <row r="407" spans="1:4" x14ac:dyDescent="0.25">
@@ -7724,10 +8050,10 @@
         <v>93</v>
       </c>
       <c r="C407" s="4" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="D407" s="5" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
     </row>
     <row r="408" spans="1:4" x14ac:dyDescent="0.25">
@@ -7738,10 +8064,10 @@
         <v>116</v>
       </c>
       <c r="C408" s="4" t="s">
+        <v>414</v>
+      </c>
+      <c r="D408" s="5" t="s">
         <v>415</v>
-      </c>
-      <c r="D408" s="5" t="s">
-        <v>416</v>
       </c>
     </row>
     <row r="409" spans="1:4" x14ac:dyDescent="0.25">
@@ -7752,7 +8078,7 @@
         <v>103</v>
       </c>
       <c r="C409" s="4" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="D409" s="5" t="s">
         <v>67</v>
@@ -7766,7 +8092,7 @@
         <v>116</v>
       </c>
       <c r="C410" s="4" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="D410" s="5" t="s">
         <v>81</v>
@@ -7780,7 +8106,7 @@
         <v>93</v>
       </c>
       <c r="C411" s="4" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="D411" s="5" t="s">
         <v>40</v>
@@ -7794,7 +8120,7 @@
         <v>305</v>
       </c>
       <c r="C412" s="4" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="D412" s="5" t="s">
         <v>199</v>
@@ -7808,7 +8134,7 @@
         <v>305</v>
       </c>
       <c r="C413" s="4" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="D413" s="5" t="s">
         <v>199</v>
@@ -7819,13 +8145,13 @@
         <v>413</v>
       </c>
       <c r="B414" s="4" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="C414" s="4" t="s">
         <v>24</v>
       </c>
       <c r="D414" s="5" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
     </row>
     <row r="415" spans="1:4" x14ac:dyDescent="0.25">
@@ -7847,10 +8173,10 @@
         <v>415</v>
       </c>
       <c r="B416" s="4" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="C416" s="4" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="D416" s="5">
         <v>82</v>
@@ -7878,7 +8204,7 @@
         <v>113</v>
       </c>
       <c r="C418" s="4" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="D418" s="5">
         <v>81</v>
@@ -7892,7 +8218,7 @@
         <v>240</v>
       </c>
       <c r="C419" s="4" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="D419" s="5">
         <v>67</v>
@@ -7906,7 +8232,7 @@
         <v>111</v>
       </c>
       <c r="C420" s="4" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="D420" s="5">
         <v>130</v>
@@ -7920,7 +8246,7 @@
         <v>111</v>
       </c>
       <c r="C421" s="4" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="D421" s="5">
         <v>67</v>
@@ -7934,7 +8260,7 @@
         <v>91</v>
       </c>
       <c r="C422" s="21" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
       <c r="D422" s="22" t="s">
         <v>56</v>
@@ -7962,7 +8288,7 @@
         <v>91</v>
       </c>
       <c r="C424" s="21" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="D424" s="22" t="s">
         <v>56</v>
@@ -7976,7 +8302,7 @@
         <v>4</v>
       </c>
       <c r="C425" s="21" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="D425" s="22" t="s">
         <v>218</v>
@@ -7990,7 +8316,7 @@
         <v>113</v>
       </c>
       <c r="C426" s="21" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
       <c r="D426" s="22" t="s">
         <v>45</v>
@@ -8004,7 +8330,7 @@
         <v>113</v>
       </c>
       <c r="C427" s="21" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="D427" s="22" t="s">
         <v>45</v>
@@ -8015,7 +8341,7 @@
         <v>427</v>
       </c>
       <c r="B428" s="21" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="C428" s="21" t="s">
         <v>8</v>
@@ -8029,10 +8355,10 @@
         <v>428</v>
       </c>
       <c r="B429" s="21" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="C429" s="21" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
       <c r="D429" s="22" t="s">
         <v>9</v>
@@ -8046,7 +8372,7 @@
         <v>91</v>
       </c>
       <c r="C430" s="21" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
       <c r="D430" s="22" t="s">
         <v>61</v>
@@ -8060,7 +8386,7 @@
         <v>93</v>
       </c>
       <c r="C431" s="21" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
       <c r="D431" s="22" t="s">
         <v>54</v>
@@ -8074,7 +8400,7 @@
         <v>246</v>
       </c>
       <c r="C432" s="21" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
       <c r="D432" s="22" t="s">
         <v>56</v>
@@ -8085,7 +8411,7 @@
         <v>432</v>
       </c>
       <c r="B433" s="21" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="C433" s="21" t="s">
         <v>102</v>
@@ -8099,7 +8425,7 @@
         <v>433</v>
       </c>
       <c r="B434" s="21" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="C434" s="21" t="s">
         <v>34</v>
@@ -8116,7 +8442,7 @@
         <v>50</v>
       </c>
       <c r="C435" s="21" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
       <c r="D435" s="22" t="s">
         <v>195</v>
@@ -8127,13 +8453,13 @@
         <v>435</v>
       </c>
       <c r="B436" s="21" t="s">
+        <v>436</v>
+      </c>
+      <c r="C436" s="21" t="s">
         <v>437</v>
       </c>
-      <c r="C436" s="21" t="s">
+      <c r="D436" s="22" t="s">
         <v>438</v>
-      </c>
-      <c r="D436" s="22" t="s">
-        <v>439</v>
       </c>
     </row>
     <row r="437" spans="1:4" x14ac:dyDescent="0.25">
@@ -8148,6 +8474,1280 @@
       </c>
       <c r="D437" s="22">
         <v>313</v>
+      </c>
+    </row>
+    <row r="438" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A438" s="20">
+        <v>437</v>
+      </c>
+      <c r="B438" s="21" t="s">
+        <v>91</v>
+      </c>
+      <c r="C438" s="21" t="s">
+        <v>439</v>
+      </c>
+      <c r="D438" s="22">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="439" spans="1:4" ht="22.5" x14ac:dyDescent="0.25">
+      <c r="A439" s="20">
+        <v>438</v>
+      </c>
+      <c r="B439" s="21" t="s">
+        <v>246</v>
+      </c>
+      <c r="C439" s="21" t="s">
+        <v>440</v>
+      </c>
+      <c r="D439" s="22">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="440" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A440" s="20">
+        <v>439</v>
+      </c>
+      <c r="B440" s="21" t="s">
+        <v>441</v>
+      </c>
+      <c r="C440" s="21" t="s">
+        <v>301</v>
+      </c>
+      <c r="D440" s="22">
+        <v>369</v>
+      </c>
+    </row>
+    <row r="441" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A441" s="20">
+        <v>440</v>
+      </c>
+      <c r="B441" s="21" t="s">
+        <v>323</v>
+      </c>
+      <c r="C441" s="21" t="s">
+        <v>442</v>
+      </c>
+      <c r="D441" s="22">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="442" spans="1:4" ht="22.5" x14ac:dyDescent="0.25">
+      <c r="A442" s="20">
+        <v>441</v>
+      </c>
+      <c r="B442" s="21" t="s">
+        <v>246</v>
+      </c>
+      <c r="C442" s="21" t="s">
+        <v>352</v>
+      </c>
+      <c r="D442" s="22">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="443" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A443" s="20">
+        <v>442</v>
+      </c>
+      <c r="B443" s="21" t="s">
+        <v>323</v>
+      </c>
+      <c r="C443" s="21" t="s">
+        <v>443</v>
+      </c>
+      <c r="D443" s="22">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="444" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A444" s="20">
+        <v>443</v>
+      </c>
+      <c r="B444" s="21" t="s">
+        <v>240</v>
+      </c>
+      <c r="C444" s="21" t="s">
+        <v>444</v>
+      </c>
+      <c r="D444" s="22">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="445" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A445" s="20">
+        <v>444</v>
+      </c>
+      <c r="B445" s="23" t="s">
+        <v>50</v>
+      </c>
+      <c r="C445" s="23" t="s">
+        <v>445</v>
+      </c>
+      <c r="D445" s="24">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="446" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A446" s="20">
+        <v>445</v>
+      </c>
+      <c r="B446" s="21" t="s">
+        <v>50</v>
+      </c>
+      <c r="C446" s="21" t="s">
+        <v>446</v>
+      </c>
+      <c r="D446" s="22">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="447" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A447" s="20">
+        <v>446</v>
+      </c>
+      <c r="B447" s="21" t="s">
+        <v>240</v>
+      </c>
+      <c r="C447" s="21" t="s">
+        <v>206</v>
+      </c>
+      <c r="D447" s="22">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="448" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A448" s="20">
+        <v>447</v>
+      </c>
+      <c r="B448" s="21" t="s">
+        <v>116</v>
+      </c>
+      <c r="C448" s="21" t="s">
+        <v>447</v>
+      </c>
+      <c r="D448" s="22">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="449" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A449" s="20">
+        <v>448</v>
+      </c>
+      <c r="B449" s="21" t="s">
+        <v>240</v>
+      </c>
+      <c r="C449" s="21" t="s">
+        <v>448</v>
+      </c>
+      <c r="D449" s="22">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="450" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A450" s="20">
+        <v>449</v>
+      </c>
+      <c r="B450" s="21" t="s">
+        <v>50</v>
+      </c>
+      <c r="C450" s="21" t="s">
+        <v>269</v>
+      </c>
+      <c r="D450" s="22">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="451" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A451" s="20">
+        <v>450</v>
+      </c>
+      <c r="B451" s="21" t="s">
+        <v>227</v>
+      </c>
+      <c r="C451" s="21" t="s">
+        <v>104</v>
+      </c>
+      <c r="D451" s="22">
+        <v>323</v>
+      </c>
+    </row>
+    <row r="452" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A452" s="20">
+        <v>451</v>
+      </c>
+      <c r="B452" s="21" t="s">
+        <v>441</v>
+      </c>
+      <c r="C452" s="21" t="s">
+        <v>69</v>
+      </c>
+      <c r="D452" s="22">
+        <v>323</v>
+      </c>
+    </row>
+    <row r="453" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A453" s="20">
+        <v>452</v>
+      </c>
+      <c r="B453" s="21" t="s">
+        <v>337</v>
+      </c>
+      <c r="C453" s="21" t="s">
+        <v>241</v>
+      </c>
+      <c r="D453" s="22" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="454" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A454" s="20">
+        <v>453</v>
+      </c>
+      <c r="B454" s="21" t="s">
+        <v>111</v>
+      </c>
+      <c r="C454" s="21" t="s">
+        <v>179</v>
+      </c>
+      <c r="D454" s="22">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="455" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A455" s="20">
+        <v>454</v>
+      </c>
+      <c r="B455" s="21" t="s">
+        <v>13</v>
+      </c>
+      <c r="C455" s="21" t="s">
+        <v>449</v>
+      </c>
+      <c r="D455" s="22">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="456" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A456" s="20">
+        <v>455</v>
+      </c>
+      <c r="B456" s="21" t="s">
+        <v>227</v>
+      </c>
+      <c r="C456" s="21" t="s">
+        <v>310</v>
+      </c>
+      <c r="D456" s="22">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="457" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A457" s="20">
+        <v>456</v>
+      </c>
+      <c r="B457" s="21" t="s">
+        <v>37</v>
+      </c>
+      <c r="C457" s="21" t="s">
+        <v>301</v>
+      </c>
+      <c r="D457" s="22" t="s">
+        <v>450</v>
+      </c>
+    </row>
+    <row r="458" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A458" s="20">
+        <v>457</v>
+      </c>
+      <c r="B458" s="21" t="s">
+        <v>37</v>
+      </c>
+      <c r="C458" s="21" t="s">
+        <v>69</v>
+      </c>
+      <c r="D458" s="22" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="459" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A459" s="20">
+        <v>458</v>
+      </c>
+      <c r="B459" s="21" t="s">
+        <v>4</v>
+      </c>
+      <c r="C459" s="21" t="s">
+        <v>451</v>
+      </c>
+      <c r="D459" s="22">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="460" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A460" s="20">
+        <v>459</v>
+      </c>
+      <c r="B460" s="21" t="s">
+        <v>7</v>
+      </c>
+      <c r="C460" s="21" t="s">
+        <v>452</v>
+      </c>
+      <c r="D460" s="22">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="461" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A461" s="20">
+        <v>460</v>
+      </c>
+      <c r="B461" s="21" t="s">
+        <v>62</v>
+      </c>
+      <c r="C461" s="21" t="s">
+        <v>304</v>
+      </c>
+      <c r="D461" s="22" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="462" spans="1:4" ht="22.5" x14ac:dyDescent="0.25">
+      <c r="A462" s="20">
+        <v>461</v>
+      </c>
+      <c r="B462" s="21" t="s">
+        <v>246</v>
+      </c>
+      <c r="C462" s="21" t="s">
+        <v>453</v>
+      </c>
+      <c r="D462" s="22" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="463" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A463" s="20">
+        <v>462</v>
+      </c>
+      <c r="B463" s="21" t="s">
+        <v>93</v>
+      </c>
+      <c r="C463" s="21" t="s">
+        <v>454</v>
+      </c>
+      <c r="D463" s="22" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="464" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A464" s="20">
+        <v>463</v>
+      </c>
+      <c r="B464" s="21" t="s">
+        <v>338</v>
+      </c>
+      <c r="C464" s="21" t="s">
+        <v>455</v>
+      </c>
+      <c r="D464" s="22" t="s">
+        <v>387</v>
+      </c>
+    </row>
+    <row r="465" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A465" s="20">
+        <v>464</v>
+      </c>
+      <c r="B465" s="21" t="s">
+        <v>93</v>
+      </c>
+      <c r="C465" s="21" t="s">
+        <v>456</v>
+      </c>
+      <c r="D465" s="22" t="s">
+        <v>387</v>
+      </c>
+    </row>
+    <row r="466" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A466" s="20">
+        <v>465</v>
+      </c>
+      <c r="B466" s="21" t="s">
+        <v>83</v>
+      </c>
+      <c r="C466" s="21" t="s">
+        <v>457</v>
+      </c>
+      <c r="D466" s="22" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="467" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A467" s="20">
+        <v>466</v>
+      </c>
+      <c r="B467" s="21" t="s">
+        <v>458</v>
+      </c>
+      <c r="C467" s="21" t="s">
+        <v>316</v>
+      </c>
+      <c r="D467" s="22" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="468" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A468" s="20">
+        <v>467</v>
+      </c>
+      <c r="B468" s="21" t="s">
+        <v>385</v>
+      </c>
+      <c r="C468" s="21" t="s">
+        <v>460</v>
+      </c>
+      <c r="D468" s="22" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="469" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A469" s="20">
+        <v>468</v>
+      </c>
+      <c r="B469" s="21" t="s">
+        <v>385</v>
+      </c>
+      <c r="C469" s="21" t="s">
+        <v>461</v>
+      </c>
+      <c r="D469" s="22" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="470" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A470" s="20">
+        <v>469</v>
+      </c>
+      <c r="B470" s="21" t="s">
+        <v>385</v>
+      </c>
+      <c r="C470" s="21" t="s">
+        <v>462</v>
+      </c>
+      <c r="D470" s="22" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="471" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A471" s="20">
+        <v>470</v>
+      </c>
+      <c r="B471" s="21" t="s">
+        <v>385</v>
+      </c>
+      <c r="C471" s="21" t="s">
+        <v>463</v>
+      </c>
+      <c r="D471" s="22" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="472" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A472" s="20">
+        <v>471</v>
+      </c>
+      <c r="B472" s="21" t="s">
+        <v>385</v>
+      </c>
+      <c r="C472" s="21" t="s">
+        <v>464</v>
+      </c>
+      <c r="D472" s="22" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="473" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A473" s="20">
+        <v>472</v>
+      </c>
+      <c r="B473" s="21" t="s">
+        <v>465</v>
+      </c>
+      <c r="C473" s="21" t="s">
+        <v>466</v>
+      </c>
+      <c r="D473" s="22" t="s">
+        <v>467</v>
+      </c>
+    </row>
+    <row r="474" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A474" s="20">
+        <v>473</v>
+      </c>
+      <c r="B474" s="21" t="s">
+        <v>465</v>
+      </c>
+      <c r="C474" s="21" t="s">
+        <v>468</v>
+      </c>
+      <c r="D474" s="22" t="s">
+        <v>469</v>
+      </c>
+    </row>
+    <row r="475" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A475" s="20">
+        <v>474</v>
+      </c>
+      <c r="B475" s="21" t="s">
+        <v>83</v>
+      </c>
+      <c r="C475" s="21" t="s">
+        <v>380</v>
+      </c>
+      <c r="D475" s="22" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="476" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A476" s="20">
+        <v>475</v>
+      </c>
+      <c r="B476" s="21" t="s">
+        <v>83</v>
+      </c>
+      <c r="C476" s="21" t="s">
+        <v>470</v>
+      </c>
+      <c r="D476" s="22" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="477" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A477" s="20">
+        <v>476</v>
+      </c>
+      <c r="B477" s="21" t="s">
+        <v>91</v>
+      </c>
+      <c r="C477" s="21" t="s">
+        <v>471</v>
+      </c>
+      <c r="D477" s="22" t="s">
+        <v>472</v>
+      </c>
+    </row>
+    <row r="478" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A478" s="20">
+        <v>477</v>
+      </c>
+      <c r="B478" s="21" t="s">
+        <v>83</v>
+      </c>
+      <c r="C478" s="21" t="s">
+        <v>473</v>
+      </c>
+      <c r="D478" s="22" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="479" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A479" s="20">
+        <v>478</v>
+      </c>
+      <c r="B479" s="21" t="s">
+        <v>83</v>
+      </c>
+      <c r="C479" s="21" t="s">
+        <v>474</v>
+      </c>
+      <c r="D479" s="22" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="480" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A480" s="20">
+        <v>479</v>
+      </c>
+      <c r="B480" s="21" t="s">
+        <v>83</v>
+      </c>
+      <c r="C480" s="21" t="s">
+        <v>475</v>
+      </c>
+      <c r="D480" s="22" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="481" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A481" s="20">
+        <v>480</v>
+      </c>
+      <c r="B481" s="21" t="s">
+        <v>116</v>
+      </c>
+      <c r="C481" s="21" t="s">
+        <v>476</v>
+      </c>
+      <c r="D481" s="22" t="s">
+        <v>477</v>
+      </c>
+    </row>
+    <row r="482" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A482" s="20">
+        <v>481</v>
+      </c>
+      <c r="B482" s="21" t="s">
+        <v>116</v>
+      </c>
+      <c r="C482" s="21" t="s">
+        <v>478</v>
+      </c>
+      <c r="D482" s="22" t="s">
+        <v>477</v>
+      </c>
+    </row>
+    <row r="483" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A483" s="20">
+        <v>482</v>
+      </c>
+      <c r="B483" s="21" t="s">
+        <v>305</v>
+      </c>
+      <c r="C483" s="21" t="s">
+        <v>479</v>
+      </c>
+      <c r="D483" s="22" t="s">
+        <v>480</v>
+      </c>
+    </row>
+    <row r="484" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A484" s="20">
+        <v>483</v>
+      </c>
+      <c r="B484" s="21" t="s">
+        <v>305</v>
+      </c>
+      <c r="C484" s="21" t="s">
+        <v>481</v>
+      </c>
+      <c r="D484" s="22" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="485" spans="1:4" ht="22.5" x14ac:dyDescent="0.25">
+      <c r="A485" s="20">
+        <v>484</v>
+      </c>
+      <c r="B485" s="21" t="s">
+        <v>246</v>
+      </c>
+      <c r="C485" s="21" t="s">
+        <v>482</v>
+      </c>
+      <c r="D485" s="22" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="486" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A486" s="20">
+        <v>485</v>
+      </c>
+      <c r="B486" s="21" t="s">
+        <v>227</v>
+      </c>
+      <c r="C486" s="21" t="s">
+        <v>483</v>
+      </c>
+      <c r="D486" s="22" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="487" spans="1:4" ht="22.5" x14ac:dyDescent="0.25">
+      <c r="A487" s="20">
+        <v>486</v>
+      </c>
+      <c r="B487" s="21" t="s">
+        <v>484</v>
+      </c>
+      <c r="C487" s="21" t="s">
+        <v>115</v>
+      </c>
+      <c r="D487" s="22" t="s">
+        <v>485</v>
+      </c>
+    </row>
+    <row r="488" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A488" s="20">
+        <v>487</v>
+      </c>
+      <c r="B488" s="21" t="s">
+        <v>240</v>
+      </c>
+      <c r="C488" s="21" t="s">
+        <v>486</v>
+      </c>
+      <c r="D488" s="22" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="489" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A489" s="20">
+        <v>488</v>
+      </c>
+      <c r="B489" s="21" t="s">
+        <v>113</v>
+      </c>
+      <c r="C489" s="21" t="s">
+        <v>52</v>
+      </c>
+      <c r="D489" s="22" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="490" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A490" s="20">
+        <v>489</v>
+      </c>
+      <c r="B490" s="21" t="s">
+        <v>487</v>
+      </c>
+      <c r="C490" s="21" t="s">
+        <v>488</v>
+      </c>
+      <c r="D490" s="22" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="491" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A491" s="20">
+        <v>490</v>
+      </c>
+      <c r="B491" s="21" t="s">
+        <v>113</v>
+      </c>
+      <c r="C491" s="21" t="s">
+        <v>489</v>
+      </c>
+      <c r="D491" s="22" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="492" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A492" s="20">
+        <v>491</v>
+      </c>
+      <c r="B492" s="21" t="s">
+        <v>91</v>
+      </c>
+      <c r="C492" s="21" t="s">
+        <v>90</v>
+      </c>
+      <c r="D492" s="22" t="s">
+        <v>490</v>
+      </c>
+    </row>
+    <row r="493" spans="1:4" ht="22.5" x14ac:dyDescent="0.25">
+      <c r="A493" s="20">
+        <v>492</v>
+      </c>
+      <c r="B493" s="21" t="s">
+        <v>246</v>
+      </c>
+      <c r="C493" s="21" t="s">
+        <v>491</v>
+      </c>
+      <c r="D493" s="22" t="s">
+        <v>492</v>
+      </c>
+    </row>
+    <row r="494" spans="1:4" ht="22.5" x14ac:dyDescent="0.25">
+      <c r="A494" s="20">
+        <v>493</v>
+      </c>
+      <c r="B494" s="21" t="s">
+        <v>246</v>
+      </c>
+      <c r="C494" s="21" t="s">
+        <v>466</v>
+      </c>
+      <c r="D494" s="22" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="495" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A495" s="20">
+        <v>494</v>
+      </c>
+      <c r="B495" s="21" t="s">
+        <v>111</v>
+      </c>
+      <c r="C495" s="21" t="s">
+        <v>493</v>
+      </c>
+      <c r="D495" s="22" t="s">
+        <v>492</v>
+      </c>
+    </row>
+    <row r="496" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A496" s="20">
+        <v>495</v>
+      </c>
+      <c r="B496" s="21" t="s">
+        <v>4</v>
+      </c>
+      <c r="C496" s="21" t="s">
+        <v>494</v>
+      </c>
+      <c r="D496" s="22" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="497" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A497" s="20">
+        <v>496</v>
+      </c>
+      <c r="B497" s="21" t="s">
+        <v>50</v>
+      </c>
+      <c r="C497" s="21" t="s">
+        <v>166</v>
+      </c>
+      <c r="D497" s="22" t="s">
+        <v>412</v>
+      </c>
+    </row>
+    <row r="498" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A498" s="20">
+        <v>497</v>
+      </c>
+      <c r="B498" s="21" t="s">
+        <v>62</v>
+      </c>
+      <c r="C498" s="21" t="s">
+        <v>495</v>
+      </c>
+      <c r="D498" s="22" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="499" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A499" s="20">
+        <v>498</v>
+      </c>
+      <c r="B499" s="21" t="s">
+        <v>227</v>
+      </c>
+      <c r="C499" s="21" t="s">
+        <v>496</v>
+      </c>
+      <c r="D499" s="22" t="s">
+        <v>497</v>
+      </c>
+    </row>
+    <row r="500" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A500" s="20">
+        <v>499</v>
+      </c>
+      <c r="B500" s="21" t="s">
+        <v>141</v>
+      </c>
+      <c r="C500" s="21" t="s">
+        <v>498</v>
+      </c>
+      <c r="D500" s="22" t="s">
+        <v>499</v>
+      </c>
+    </row>
+    <row r="501" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A501" s="20">
+        <v>500</v>
+      </c>
+      <c r="B501" s="21" t="s">
+        <v>7</v>
+      </c>
+      <c r="C501" s="21" t="s">
+        <v>500</v>
+      </c>
+      <c r="D501" s="22">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="502" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A502" s="20">
+        <v>501</v>
+      </c>
+      <c r="B502" s="21" t="s">
+        <v>113</v>
+      </c>
+      <c r="C502" s="21" t="s">
+        <v>501</v>
+      </c>
+      <c r="D502" s="22">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="503" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A503" s="20">
+        <v>502</v>
+      </c>
+      <c r="B503" s="21" t="s">
+        <v>502</v>
+      </c>
+      <c r="C503" s="21" t="s">
+        <v>503</v>
+      </c>
+      <c r="D503" s="22" t="s">
+        <v>504</v>
+      </c>
+    </row>
+    <row r="504" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A504" s="20">
+        <v>503</v>
+      </c>
+      <c r="B504" s="21" t="s">
+        <v>240</v>
+      </c>
+      <c r="C504" s="21" t="s">
+        <v>505</v>
+      </c>
+      <c r="D504" s="22" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="505" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A505" s="20">
+        <v>504</v>
+      </c>
+      <c r="B505" s="21" t="s">
+        <v>93</v>
+      </c>
+      <c r="C505" s="21" t="s">
+        <v>506</v>
+      </c>
+      <c r="D505" s="22" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="506" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A506" s="20">
+        <v>505</v>
+      </c>
+      <c r="B506" s="21" t="s">
+        <v>93</v>
+      </c>
+      <c r="C506" s="21" t="s">
+        <v>507</v>
+      </c>
+      <c r="D506" s="22" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="507" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A507" s="20">
+        <v>506</v>
+      </c>
+      <c r="B507" s="21" t="s">
+        <v>337</v>
+      </c>
+      <c r="C507" s="21" t="s">
+        <v>508</v>
+      </c>
+      <c r="D507" s="22">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="508" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A508" s="20">
+        <v>507</v>
+      </c>
+      <c r="B508" s="21" t="s">
+        <v>83</v>
+      </c>
+      <c r="C508" s="21" t="s">
+        <v>356</v>
+      </c>
+      <c r="D508" s="22">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="509" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A509" s="20">
+        <v>508</v>
+      </c>
+      <c r="B509" s="21" t="s">
+        <v>240</v>
+      </c>
+      <c r="C509" s="21" t="s">
+        <v>509</v>
+      </c>
+      <c r="D509" s="22">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="510" spans="1:4" ht="22.5" x14ac:dyDescent="0.25">
+      <c r="A510" s="20">
+        <v>509</v>
+      </c>
+      <c r="B510" s="21" t="s">
+        <v>510</v>
+      </c>
+      <c r="C510" s="21" t="s">
+        <v>451</v>
+      </c>
+      <c r="D510" s="22">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="511" spans="1:4" ht="22.5" x14ac:dyDescent="0.25">
+      <c r="A511" s="20">
+        <v>510</v>
+      </c>
+      <c r="B511" s="21" t="s">
+        <v>510</v>
+      </c>
+      <c r="C511" s="21" t="s">
+        <v>454</v>
+      </c>
+      <c r="D511" s="22">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="512" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A512" s="20">
+        <v>511</v>
+      </c>
+      <c r="B512" s="21" t="s">
+        <v>113</v>
+      </c>
+      <c r="C512" s="21" t="s">
+        <v>511</v>
+      </c>
+      <c r="D512" s="22">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="513" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A513" s="20">
+        <v>512</v>
+      </c>
+      <c r="B513" s="21" t="s">
+        <v>111</v>
+      </c>
+      <c r="C513" s="21" t="s">
+        <v>249</v>
+      </c>
+      <c r="D513" s="22">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="514" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A514" s="20">
+        <v>513</v>
+      </c>
+      <c r="B514" s="21" t="s">
+        <v>93</v>
+      </c>
+      <c r="C514" s="21" t="s">
+        <v>288</v>
+      </c>
+      <c r="D514" s="22">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="515" spans="1:4" ht="22.5" x14ac:dyDescent="0.25">
+      <c r="A515" s="20">
+        <v>514</v>
+      </c>
+      <c r="B515" s="21" t="s">
+        <v>246</v>
+      </c>
+      <c r="C515" s="21" t="s">
+        <v>512</v>
+      </c>
+      <c r="D515" s="22">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="516" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A516" s="25">
+        <v>515</v>
+      </c>
+      <c r="B516" s="26" t="s">
+        <v>13</v>
+      </c>
+      <c r="C516" s="26" t="s">
+        <v>513</v>
+      </c>
+      <c r="D516" s="27" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="517" spans="1:4" ht="22.5" x14ac:dyDescent="0.25">
+      <c r="A517" s="20">
+        <v>516</v>
+      </c>
+      <c r="B517" s="21" t="s">
+        <v>37</v>
+      </c>
+      <c r="C517" s="21" t="s">
+        <v>514</v>
+      </c>
+      <c r="D517" s="22">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="518" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A518" s="20">
+        <v>517</v>
+      </c>
+      <c r="B518" s="21" t="s">
+        <v>13</v>
+      </c>
+      <c r="C518" s="21" t="s">
+        <v>515</v>
+      </c>
+      <c r="D518" s="22">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="519" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A519" s="20">
+        <v>518</v>
+      </c>
+      <c r="B519" s="21" t="s">
+        <v>113</v>
+      </c>
+      <c r="C519" s="21" t="s">
+        <v>254</v>
+      </c>
+      <c r="D519" s="22" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="520" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A520" s="20">
+        <v>519</v>
+      </c>
+      <c r="B520" s="21" t="s">
+        <v>50</v>
+      </c>
+      <c r="C520" s="21" t="s">
+        <v>516</v>
+      </c>
+      <c r="D520" s="22">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="521" spans="1:4" ht="22.5" x14ac:dyDescent="0.25">
+      <c r="A521" s="20">
+        <v>520</v>
+      </c>
+      <c r="B521" s="21" t="s">
+        <v>93</v>
+      </c>
+      <c r="C521" s="21" t="s">
+        <v>226</v>
+      </c>
+      <c r="D521" s="22">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="522" spans="1:4" ht="22.5" x14ac:dyDescent="0.25">
+      <c r="A522" s="20">
+        <v>521</v>
+      </c>
+      <c r="B522" s="21" t="s">
+        <v>246</v>
+      </c>
+      <c r="C522" s="21" t="s">
+        <v>299</v>
+      </c>
+      <c r="D522" s="22">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="523" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A523" s="20">
+        <v>522</v>
+      </c>
+      <c r="B523" s="21" t="s">
+        <v>4</v>
+      </c>
+      <c r="C523" s="21" t="s">
+        <v>517</v>
+      </c>
+      <c r="D523" s="22">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="524" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A524" s="20">
+        <v>523</v>
+      </c>
+      <c r="B524" s="21" t="s">
+        <v>518</v>
+      </c>
+      <c r="C524" s="21" t="s">
+        <v>483</v>
+      </c>
+      <c r="D524" s="22">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="525" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A525" s="20">
+        <v>524</v>
+      </c>
+      <c r="B525" s="21" t="s">
+        <v>93</v>
+      </c>
+      <c r="C525" s="21" t="s">
+        <v>519</v>
+      </c>
+      <c r="D525" s="22" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="526" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A526" s="20">
+        <v>525</v>
+      </c>
+      <c r="B526" s="21" t="s">
+        <v>93</v>
+      </c>
+      <c r="C526" s="21" t="s">
+        <v>51</v>
+      </c>
+      <c r="D526" s="22" t="s">
+        <v>412</v>
+      </c>
+    </row>
+    <row r="527" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A527" s="28">
+        <v>526</v>
+      </c>
+      <c r="B527" s="29" t="s">
+        <v>4</v>
+      </c>
+      <c r="C527" s="29" t="s">
+        <v>520</v>
+      </c>
+      <c r="D527" s="30" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="528" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A528" s="28">
+        <v>527</v>
+      </c>
+      <c r="B528" s="29" t="s">
+        <v>307</v>
+      </c>
+      <c r="C528" s="29" t="s">
+        <v>521</v>
+      </c>
+      <c r="D528" s="30">
+        <v>123</v>
       </c>
     </row>
   </sheetData>

</xml_diff>